<commit_message>
FLiBe Testing (very good)
</commit_message>
<xml_diff>
--- a/OpenMC_STAR_Model/TBR's.xlsx
+++ b/OpenMC_STAR_Model/TBR's.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rocco698/Desktop/Undergrad/Spring_2026/NUCE_431W/NUCE_431W/OpenMC_STAR_Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{878D8CFE-8507-C446-9345-141578531E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614CD86B-93E0-444B-9B4E-B70BA37C1B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{19FD8DC0-BE1F-DA49-9BCD-F45CFD8ECFC9}"/>
+    <workbookView minimized="1" xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{19FD8DC0-BE1F-DA49-9BCD-F45CFD8ECFC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,6 +33,20 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>Material</t>
+  </si>
+  <si>
+    <t>(n,t)</t>
+  </si>
+  <si>
+    <t>PbLi (nat.)</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -402,9 +416,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21FEB923-94CE-9048-A235-5E054F03F29C}">
-  <dimension ref="A1"/>
+  <dimension ref="A2:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>0.42057800000000001</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Further TBR Testing and Benchmarking
</commit_message>
<xml_diff>
--- a/OpenMC_STAR_Model/TBR's.xlsx
+++ b/OpenMC_STAR_Model/TBR's.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rocco698/Desktop/Undergrad/Spring_2026/NUCE_431W/NUCE_431W/OpenMC_STAR_Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614CD86B-93E0-444B-9B4E-B70BA37C1B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0461AA94-25D9-C348-B045-7CB502B5C13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{19FD8DC0-BE1F-DA49-9BCD-F45CFD8ECFC9}"/>
+    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{19FD8DC0-BE1F-DA49-9BCD-F45CFD8ECFC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,15 +36,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>Material</t>
-  </si>
-  <si>
-    <t>(n,t)</t>
-  </si>
-  <si>
-    <t>PbLi (nat.)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="9">
+  <si>
+    <t>Particles</t>
+  </si>
+  <si>
+    <t>at % Li</t>
+  </si>
+  <si>
+    <t>FLiBe</t>
+  </si>
+  <si>
+    <t>10K</t>
+  </si>
+  <si>
+    <t>TBR (n,Xt)</t>
+  </si>
+  <si>
+    <t>Margin</t>
+  </si>
+  <si>
+    <t>PbLi (Natural Li, 9.5 gcc)</t>
+  </si>
+  <si>
+    <t>FLiNaK</t>
+  </si>
+  <si>
+    <t>Density (g/cc)</t>
   </si>
 </sst>
 </file>
@@ -80,8 +98,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,23 +435,122 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21FEB923-94CE-9048-A235-5E054F03F29C}">
-  <dimension ref="A2:B3"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
       </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s">
+        <v>4</v>
+      </c>
+      <c r="M2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3">
-        <v>0.42057800000000001</v>
+        <v>0.17</v>
+      </c>
+      <c r="C3">
+        <v>0.44600200000000001</v>
+      </c>
+      <c r="D3">
+        <v>1.4223599999999999E-3</v>
+      </c>
+      <c r="E3">
+        <v>9.5</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3">
+        <v>1.0445199999999999</v>
+      </c>
+      <c r="I3">
+        <v>3.1094999999999999E-3</v>
+      </c>
+      <c r="K3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <v>0.86896099999999998</v>
+      </c>
+      <c r="M3">
+        <v>3.05902E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="C4">
+        <v>1.0500100000000001</v>
+      </c>
+      <c r="D4">
+        <v>2.3920299999999999E-3</v>
+      </c>
+      <c r="E4">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1.0569999999999999</v>
+      </c>
+      <c r="D5">
+        <v>2.09756E-3</v>
+      </c>
+      <c r="E5">
+        <v>0.51200000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Additional Material Testing For TBR
</commit_message>
<xml_diff>
--- a/OpenMC_STAR_Model/TBR's.xlsx
+++ b/OpenMC_STAR_Model/TBR's.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Leaft\Desktop\Temp. Hw\Capstone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rocco698/Desktop/Undergrad/Spring_2026/NUCE_431W/NUCE_431W/OpenMC_STAR_Model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2BCF699-029F-49BA-A9CE-3EB09102720A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E0ADD66-87CA-E544-9681-F872AE0106B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{19FD8DC0-BE1F-DA49-9BCD-F45CFD8ECFC9}"/>
+    <workbookView xWindow="160" yWindow="920" windowWidth="29920" windowHeight="17280" xr2:uid="{19FD8DC0-BE1F-DA49-9BCD-F45CFD8ECFC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Material" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="26">
   <si>
     <t>Particles</t>
   </si>
@@ -109,13 +109,19 @@
   </si>
   <si>
     <t>Li2TiO3</t>
+  </si>
+  <si>
+    <t>density</t>
+  </si>
+  <si>
+    <t>(nat. Li)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -123,16 +129,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -191,53 +210,37 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </left>
-      <right/>
-      <top/>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Calculation" xfId="1" builtinId="22"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -570,10 +573,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21FEB923-94CE-9048-A235-5E054F03F29C}">
-  <dimension ref="A1:Q21"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:R21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -586,10 +589,12 @@
       <c r="O1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="P1" s="4"/>
+      <c r="P1" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="Q1" s="5"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -626,14 +631,17 @@
       <c r="O2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="P2" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="Q2" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R2" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -667,11 +675,20 @@
       <c r="M3">
         <v>3.05902E-3</v>
       </c>
-      <c r="O3" s="2"/>
-      <c r="P3" s="6"/>
-      <c r="Q3" s="7"/>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="O3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="P3" s="8">
+        <v>0.89361299999999999</v>
+      </c>
+      <c r="Q3" s="8">
+        <v>3.06895E-3</v>
+      </c>
+      <c r="R3" s="8">
+        <v>2.39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -693,7 +710,7 @@
       <c r="P4" s="4"/>
       <c r="Q4" s="5"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -712,132 +729,204 @@
       <c r="O5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P5" s="6" t="s">
+      <c r="P5" t="s">
         <v>4</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="Q5" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="O6" s="8"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="10"/>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R5" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="O6" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="P6" s="8">
+        <v>1.0584899999999999</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>3.0057999999999999E-3</v>
+      </c>
+      <c r="R6" s="8">
+        <v>2.58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="O7" s="3" t="s">
         <v>19</v>
       </c>
       <c r="P7" s="4"/>
       <c r="Q7" s="5"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="O8" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P8" s="6" t="s">
+      <c r="P8" t="s">
         <v>4</v>
       </c>
-      <c r="Q8" s="7" t="s">
+      <c r="Q8" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="O9" s="8"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="10"/>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="O9" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="P9" s="8">
+        <v>1.2262500000000001</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>2.5111700000000001E-3</v>
+      </c>
+      <c r="R9" s="8">
+        <v>2.0129999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="O10" s="3" t="s">
         <v>20</v>
       </c>
       <c r="P10" s="4"/>
       <c r="Q10" s="5"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="O11" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P11" s="6" t="s">
+      <c r="P11" t="s">
         <v>4</v>
       </c>
-      <c r="Q11" s="7" t="s">
+      <c r="Q11" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="O12" s="8"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="10"/>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="O12" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="P12" s="8">
+        <v>0.69713599999999998</v>
+      </c>
+      <c r="Q12" s="8">
+        <v>2.8363199999999998E-3</v>
+      </c>
+      <c r="R12" s="8">
+        <v>2.62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="O13" s="3" t="s">
         <v>21</v>
       </c>
       <c r="P13" s="4"/>
       <c r="Q13" s="5"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="O14" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P14" s="6" t="s">
+      <c r="P14" t="s">
         <v>4</v>
       </c>
-      <c r="Q14" s="7" t="s">
+      <c r="Q14" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="O15" s="8"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="10"/>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="R14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="O15" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="P15" s="8">
+        <v>0.98226999999999998</v>
+      </c>
+      <c r="Q15" s="8">
+        <v>3.8548100000000002E-3</v>
+      </c>
+      <c r="R15" s="8">
+        <v>2.17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="O16" s="3" t="s">
         <v>22</v>
       </c>
       <c r="P16" s="4"/>
       <c r="Q16" s="5"/>
     </row>
-    <row r="17" spans="15:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="15:18" x14ac:dyDescent="0.2">
       <c r="O17" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P17" s="6" t="s">
+      <c r="P17" t="s">
         <v>4</v>
       </c>
-      <c r="Q17" s="7" t="s">
+      <c r="Q17" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="18" spans="15:17" x14ac:dyDescent="0.3">
-      <c r="O18" s="8"/>
-      <c r="P18" s="9"/>
-      <c r="Q18" s="10"/>
-    </row>
-    <row r="19" spans="15:17" x14ac:dyDescent="0.3">
+      <c r="R17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="15:18" x14ac:dyDescent="0.2">
+      <c r="O18" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="P18" s="8">
+        <v>0.93399699999999997</v>
+      </c>
+      <c r="Q18" s="8">
+        <v>2.8539099999999999E-3</v>
+      </c>
+      <c r="R18" s="8">
+        <v>4.1500000000000004</v>
+      </c>
+    </row>
+    <row r="19" spans="15:18" x14ac:dyDescent="0.2">
       <c r="O19" s="3" t="s">
         <v>23</v>
       </c>
       <c r="P19" s="4"/>
       <c r="Q19" s="5"/>
     </row>
-    <row r="20" spans="15:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="15:18" x14ac:dyDescent="0.2">
       <c r="O20" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="P20" s="6" t="s">
+      <c r="P20" t="s">
         <v>4</v>
       </c>
-      <c r="Q20" s="7" t="s">
+      <c r="Q20" s="6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="21" spans="15:17" x14ac:dyDescent="0.3">
-      <c r="O21" s="8"/>
-      <c r="P21" s="9"/>
-      <c r="Q21" s="10"/>
+      <c r="R20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="15:18" x14ac:dyDescent="0.2">
+      <c r="O21" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="P21" s="8">
+        <v>0.89149800000000001</v>
+      </c>
+      <c r="Q21" s="8">
+        <v>2.0768200000000001E-3</v>
+      </c>
+      <c r="R21" s="8">
+        <v>3.43</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -847,17 +936,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95316306-EFB9-4052-9201-767301A3C05F}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="8.796875" style="2"/>
-    <col min="4" max="4" width="8.796875" style="2"/>
-    <col min="6" max="6" width="8.796875" style="2"/>
-    <col min="7" max="7" width="9.19921875" customWidth="1"/>
-    <col min="8" max="8" width="8.796875" style="2"/>
-    <col min="11" max="11" width="8.796875" style="2"/>
+    <col min="2" max="2" width="8.83203125" style="2"/>
+    <col min="4" max="4" width="8.83203125" style="2"/>
+    <col min="6" max="6" width="8.83203125" style="2"/>
+    <col min="7" max="7" width="9.1640625" customWidth="1"/>
+    <col min="8" max="8" width="8.83203125" style="2"/>
+    <col min="11" max="11" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
@@ -874,7 +963,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -894,7 +983,7 @@
         <v>1.0569999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="F3" s="2" t="s">
         <v>12</v>
       </c>

</xml_diff>